<commit_message>
Rehire Hungary And Future Dated Hires Xpath Added
</commit_message>
<xml_diff>
--- a/Data/Hires/testDataHungry.xlsx
+++ b/Data/Hires/testDataHungry.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E0A6E8-9BBB-483F-88A6-DDE9FE190C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="177">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -382,7 +396,7 @@
     <t>Automation Comments here….</t>
   </si>
   <si>
-    <t xml:space="preserve">94 Retail Operatives </t>
+    <t>94 Retail Operatives </t>
   </si>
   <si>
     <t>16 Men’s Accessories</t>
@@ -407,9 +421,6 @@
     <t>Social Security</t>
   </si>
   <si>
-    <t>666661280</t>
-  </si>
-  <si>
     <t>01/01/2000</t>
   </si>
   <si>
@@ -506,7 +517,7 @@
     <t>IRREGULAR - Irregular Shift Pattern (Hungary Regular &amp; Irregular Shift Pattern-Hungary)</t>
   </si>
   <si>
-    <t xml:space="preserve">92 Retail Management </t>
+    <t>92 Retail Management </t>
   </si>
   <si>
     <t>251 Management Retail</t>
@@ -515,9 +526,6 @@
     <t>Social Security (TAJ) Number</t>
   </si>
   <si>
-    <t>666661281</t>
-  </si>
-  <si>
     <t>Female</t>
   </si>
   <si>
@@ -534,62 +542,86 @@
   </si>
   <si>
     <t>Mammy</t>
+  </si>
+  <si>
+    <t>666661300</t>
+  </si>
+  <si>
+    <t>666661301</t>
+  </si>
+  <si>
+    <t>666661302</t>
+  </si>
+  <si>
+    <t>666661303</t>
+  </si>
+  <si>
+    <t>666661304</t>
+  </si>
+  <si>
+    <t>666661305</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FFFF0000"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -601,13 +633,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.5999938962981048"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -633,65 +665,107 @@
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -818,9 +892,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1102,9 +1173,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CW4"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:CW7"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.6328125" customWidth="1"/>
     <col min="2" max="2" width="57.6328125" customWidth="1"/>
@@ -1157,7 +1228,7 @@
     <col min="100" max="100" width="20.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="51" customHeight="1" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:101" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1460,7 +1531,7 @@
       </c>
       <c r="CW1" s="12"/>
     </row>
-    <row r="2" ht="87.5" customHeight="1" spans="1:100" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:101" ht="87.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>95</v>
       </c>
@@ -1492,8 +1563,8 @@
         <v>104</v>
       </c>
       <c r="K2" s="20">
-        <f t="shared" ref="K2:K3" si="0">TODAY()-31</f>
-        <v>45795</v>
+        <f t="shared" ref="K2:K7" ca="1" si="0">TODAY()-31</f>
+        <v>45803</v>
       </c>
       <c r="L2" s="21" t="s">
         <v>99</v>
@@ -1535,8 +1606,8 @@
         <v>104</v>
       </c>
       <c r="Y2" s="20">
-        <f t="shared" ref="Y2:Y3" si="1">K2</f>
-        <v>45795</v>
+        <f t="shared" ref="Y2:Y3" ca="1" si="1">K2</f>
+        <v>45803</v>
       </c>
       <c r="Z2" s="19" t="s">
         <v>114</v>
@@ -1569,12 +1640,12 @@
         <v>120</v>
       </c>
       <c r="AJ2" s="32">
-        <f>TODAY()+365</f>
-        <v>46191</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46199</v>
       </c>
       <c r="AK2" s="32">
-        <f t="shared" ref="AK2:AK3" si="2">Y2+90</f>
-        <v>45885</v>
+        <f t="shared" ref="AK2:AK3" ca="1" si="2">Y2+90</f>
+        <v>45893</v>
       </c>
       <c r="AL2" s="19" t="s">
         <v>121</v>
@@ -1611,16 +1682,16 @@
         <v>128</v>
       </c>
       <c r="AW2" s="35">
-        <f t="shared" ref="AW2:AW3" si="3">Y2-1</f>
-        <v>45794</v>
+        <f t="shared" ref="AW2:AW3" ca="1" si="3">Y2-1</f>
+        <v>45802</v>
       </c>
       <c r="AX2" s="35">
-        <f t="shared" ref="AX2:AX3" si="4">Y2-1</f>
-        <v>45794</v>
+        <f t="shared" ref="AX2:AX3" ca="1" si="4">Y2-1</f>
+        <v>45802</v>
       </c>
       <c r="AY2" s="36">
-        <f t="shared" ref="AY2:AY3" si="5">AJ2</f>
-        <v>46191</v>
+        <f t="shared" ref="AY2:AY3" ca="1" si="5">AJ2</f>
+        <v>46199</v>
       </c>
       <c r="AZ2" s="25" t="s">
         <v>99</v>
@@ -1629,22 +1700,22 @@
         <v>129</v>
       </c>
       <c r="BB2" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC2" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="BC2" s="26" t="s">
+      <c r="BD2" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="BD2" s="26" t="s">
+      <c r="BE2" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF2" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="BE2" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="BF2" s="25" t="s">
-        <v>133</v>
-      </c>
       <c r="BG2" s="38">
-        <v>5555005382</v>
+        <v>5555005400</v>
       </c>
       <c r="BH2" s="26">
         <v>36526</v>
@@ -1653,10 +1724,10 @@
         <v>51136</v>
       </c>
       <c r="BJ2" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK2" s="30" t="s">
         <v>134</v>
-      </c>
-      <c r="BK2" s="30" t="s">
-        <v>135</v>
       </c>
       <c r="BL2" s="39">
         <v>32875</v>
@@ -1668,13 +1739,13 @@
         <v>111</v>
       </c>
       <c r="BO2" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP2" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ2" s="25" t="s">
         <v>136</v>
-      </c>
-      <c r="BP2" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="BQ2" s="25" t="s">
-        <v>137</v>
       </c>
       <c r="BR2" s="25" t="s">
         <v>99</v>
@@ -1686,64 +1757,64 @@
         <v>115</v>
       </c>
       <c r="BU2" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV2" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="BV2" s="41" t="s">
+      <c r="BW2" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="BW2" s="25" t="s">
+      <c r="BX2" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="BX2" s="19" t="s">
+      <c r="BY2" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="BY2" s="25" t="s">
+      <c r="BZ2" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="BZ2" s="25" t="s">
+      <c r="CA2" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="CA2" s="25" t="s">
+      <c r="CB2" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="CB2" s="25" t="s">
+      <c r="CC2" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD2" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="CE2" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF2" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="CC2" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="CD2" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="CE2" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="CF2" s="25" t="s">
+      <c r="CG2" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="CG2" s="25" t="s">
-        <v>147</v>
-      </c>
       <c r="CH2" s="25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="CI2" s="43">
         <v>100</v>
       </c>
       <c r="CJ2" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK2" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="CK2" s="25" t="s">
+      <c r="CL2" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="CM2" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="CL2" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="CM2" s="25" t="s">
+      <c r="CN2" s="25" t="s">
         <v>150</v>
-      </c>
-      <c r="CN2" s="25" t="s">
-        <v>151</v>
       </c>
       <c r="CO2" s="31" t="s">
         <v>115</v>
@@ -1770,27 +1841,27 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" ht="72.5" customHeight="1" spans="1:100" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:101" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="45" t="s">
         <v>152</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>153</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>97</v>
       </c>
       <c r="D3" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="F3" s="17" t="s">
+      <c r="G3" s="17" t="s">
         <v>155</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>156</v>
       </c>
       <c r="H3" s="18" t="s">
         <v>102</v>
@@ -1802,8 +1873,8 @@
         <v>104</v>
       </c>
       <c r="K3" s="20">
-        <f t="shared" si="0"/>
-        <v>45795</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45803</v>
       </c>
       <c r="L3" s="21" t="s">
         <v>99</v>
@@ -1812,7 +1883,7 @@
         <v>105</v>
       </c>
       <c r="N3" s="19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O3" s="23" t="s">
         <v>107</v>
@@ -1845,23 +1916,23 @@
         <v>104</v>
       </c>
       <c r="Y3" s="20">
-        <f t="shared" si="1"/>
-        <v>45795</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45803</v>
       </c>
       <c r="Z3" s="19" t="s">
         <v>114</v>
       </c>
       <c r="AA3" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB3" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="AB3" s="33" t="s">
+      <c r="AC3" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="AC3" s="30" t="s">
+      <c r="AD3" s="31" t="s">
         <v>160</v>
-      </c>
-      <c r="AD3" s="31" t="s">
-        <v>161</v>
       </c>
       <c r="AE3" s="21">
         <v>846</v>
@@ -1873,7 +1944,7 @@
         <v>10</v>
       </c>
       <c r="AH3" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AI3" s="21" t="s">
         <v>120</v>
@@ -1882,17 +1953,17 @@
         <v>115</v>
       </c>
       <c r="AK3" s="32">
-        <f t="shared" si="2"/>
-        <v>45885</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45893</v>
       </c>
       <c r="AL3" s="19" t="s">
         <v>121</v>
       </c>
       <c r="AM3" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN3" s="41" t="s">
         <v>163</v>
-      </c>
-      <c r="AN3" s="41" t="s">
-        <v>164</v>
       </c>
       <c r="AO3" s="19" t="s">
         <v>124</v>
@@ -1920,12 +1991,12 @@
         <v>128</v>
       </c>
       <c r="AW3" s="35">
-        <f t="shared" si="3"/>
-        <v>45794</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45802</v>
       </c>
       <c r="AX3" s="35">
-        <f t="shared" si="4"/>
-        <v>45794</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45802</v>
       </c>
       <c r="AY3" s="48" t="str">
         <f t="shared" si="5"/>
@@ -1935,10 +2006,10 @@
         <v>99</v>
       </c>
       <c r="BA3" s="25" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="BB3" s="37" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="BC3" s="26">
         <v>36526</v>
@@ -1950,10 +2021,10 @@
         <v>99</v>
       </c>
       <c r="BF3" s="25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BG3" s="38">
-        <v>5555005383</v>
+        <v>5555005401</v>
       </c>
       <c r="BH3" s="26">
         <v>36526</v>
@@ -1962,10 +2033,10 @@
         <v>51136</v>
       </c>
       <c r="BJ3" s="21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="BK3" s="30" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="BL3" s="39">
         <v>32875</v>
@@ -1977,13 +2048,13 @@
         <v>111</v>
       </c>
       <c r="BO3" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP3" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ3" s="25" t="s">
         <v>136</v>
-      </c>
-      <c r="BP3" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="BQ3" s="25" t="s">
-        <v>137</v>
       </c>
       <c r="BR3" s="25" t="s">
         <v>99</v>
@@ -1995,70 +2066,70 @@
         <v>115</v>
       </c>
       <c r="BU3" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV3" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="BV3" s="41" t="s">
+      <c r="BW3" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="BW3" s="25" t="s">
+      <c r="BX3" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="BY3" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="BZ3" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="CA3" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="CB3" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="CC3" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD3" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="BX3" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="BY3" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="BZ3" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="CA3" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="CB3" s="25" t="s">
+      <c r="CE3" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF3" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="CC3" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="CD3" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="CE3" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="CF3" s="25" t="s">
+      <c r="CG3" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="CG3" s="25" t="s">
-        <v>147</v>
-      </c>
       <c r="CH3" s="25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="CI3" s="43">
         <v>100</v>
       </c>
       <c r="CJ3" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK3" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="CK3" s="25" t="s">
-        <v>149</v>
-      </c>
       <c r="CL3" s="25" t="s">
         <v>99</v>
       </c>
       <c r="CM3" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="CN3" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="CO3" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="CP3" s="31" t="s">
         <v>169</v>
-      </c>
-      <c r="CN3" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="CO3" s="33" t="s">
-        <v>170</v>
-      </c>
-      <c r="CP3" s="31" t="s">
-        <v>171</v>
       </c>
       <c r="CQ3" s="44" t="s">
         <v>111</v>
@@ -2067,7 +2138,7 @@
         <v>31048</v>
       </c>
       <c r="CS3" s="31" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="CT3" s="43">
         <v>1234011</v>
@@ -2079,56 +2150,1227 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="14.5" customHeight="1" spans="36:36" x14ac:dyDescent="0.25">
-      <c r="AJ4" s="51"/>
+    <row r="4" spans="1:101" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="20">
+        <f t="shared" ca="1" si="0"/>
+        <v>45803</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="N4" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="O4" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="P4" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q4" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="S4" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="T4" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="U4" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="V4" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="W4" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="X4" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y4" s="20">
+        <f t="shared" ref="Y4:Y7" ca="1" si="7">K4</f>
+        <v>45803</v>
+      </c>
+      <c r="Z4" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA4" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB4" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="AC4" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD4" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE4" s="21">
+        <v>846</v>
+      </c>
+      <c r="AF4" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG4" s="30">
+        <v>40</v>
+      </c>
+      <c r="AH4" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="AI4" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ4" s="32">
+        <f ca="1">TODAY()+365</f>
+        <v>46199</v>
+      </c>
+      <c r="AK4" s="32">
+        <f t="shared" ref="AK4:AK7" ca="1" si="8">Y4+90</f>
+        <v>45893</v>
+      </c>
+      <c r="AL4" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="AM4" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="AN4" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO4" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="AP4" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="AQ4" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR4" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="AS4" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="AT4" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AU4" s="34" t="str">
+        <f>AB4</f>
+        <v>Fixed Term (Fixed Term)</v>
+      </c>
+      <c r="AV4" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW4" s="35">
+        <f t="shared" ref="AW4:AW7" ca="1" si="9">Y4-1</f>
+        <v>45802</v>
+      </c>
+      <c r="AX4" s="35">
+        <f t="shared" ref="AX4:AX7" ca="1" si="10">Y4-1</f>
+        <v>45802</v>
+      </c>
+      <c r="AY4" s="36">
+        <f t="shared" ref="AY4:AY7" ca="1" si="11">AJ4</f>
+        <v>46199</v>
+      </c>
+      <c r="AZ4" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA4" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="BB4" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="BC4" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="BD4" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="BE4" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF4" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="BG4" s="38">
+        <v>5555005402</v>
+      </c>
+      <c r="BH4" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BI4" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BJ4" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK4" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="BL4" s="39">
+        <v>32875</v>
+      </c>
+      <c r="BM4" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="BN4" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="BO4" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP4" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ4" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="BR4" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BS4" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="BT4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="BU4" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV4" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="BW4" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="BX4" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="BY4" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="BZ4" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="CA4" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="CB4" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="CC4" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD4" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="CE4" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF4" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CG4" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH4" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CI4" s="43">
+        <v>100</v>
+      </c>
+      <c r="CJ4" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK4" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="CL4" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="CM4" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="CN4" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="CO4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CP4" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="CQ4" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="CR4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CS4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CT4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CU4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CV4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:101" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="K5" s="20">
+        <f t="shared" ca="1" si="0"/>
+        <v>45803</v>
+      </c>
+      <c r="L5" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="N5" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="O5" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="P5" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q5" s="19">
+        <v>123</v>
+      </c>
+      <c r="R5" s="19">
+        <v>1046</v>
+      </c>
+      <c r="S5" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="T5" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="U5" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="V5" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="W5" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="X5" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y5" s="20">
+        <f t="shared" ca="1" si="7"/>
+        <v>45803</v>
+      </c>
+      <c r="Z5" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA5" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB5" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="AC5" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="AD5" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE5" s="21">
+        <v>846</v>
+      </c>
+      <c r="AF5" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG5" s="30">
+        <v>10</v>
+      </c>
+      <c r="AH5" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="AI5" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ5" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="AK5" s="32">
+        <f t="shared" ca="1" si="8"/>
+        <v>45893</v>
+      </c>
+      <c r="AL5" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="AM5" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN5" s="41" t="s">
+        <v>163</v>
+      </c>
+      <c r="AO5" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="AP5" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="AQ5" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR5" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="AS5" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="AT5" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AU5" s="33" t="str">
+        <f t="shared" ref="AU5" si="12">AB5</f>
+        <v>Permanent</v>
+      </c>
+      <c r="AV5" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW5" s="35">
+        <f t="shared" ca="1" si="9"/>
+        <v>45802</v>
+      </c>
+      <c r="AX5" s="35">
+        <f t="shared" ca="1" si="10"/>
+        <v>45802</v>
+      </c>
+      <c r="AY5" s="48" t="str">
+        <f t="shared" si="11"/>
+        <v>N/A</v>
+      </c>
+      <c r="AZ5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA5" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="BB5" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="BC5" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BD5" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BE5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF5" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="BG5" s="38">
+        <v>5555005403</v>
+      </c>
+      <c r="BH5" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BI5" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BJ5" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK5" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="BL5" s="39">
+        <v>32875</v>
+      </c>
+      <c r="BM5" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="BN5" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="BO5" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP5" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ5" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="BR5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BS5" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="BT5" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="BU5" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV5" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="BW5" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="BX5" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="BY5" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="BZ5" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="CA5" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="CB5" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="CC5" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD5" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="CE5" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF5" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CG5" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH5" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CI5" s="43">
+        <v>100</v>
+      </c>
+      <c r="CJ5" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK5" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="CL5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="CM5" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="CN5" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="CO5" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="CP5" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="CQ5" s="44" t="s">
+        <v>111</v>
+      </c>
+      <c r="CR5" s="50">
+        <v>31048</v>
+      </c>
+      <c r="CS5" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="CT5" s="43">
+        <v>1234011</v>
+      </c>
+      <c r="CU5" s="43">
+        <v>123456011</v>
+      </c>
+      <c r="CV5" s="43">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:101" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="K6" s="20">
+        <f t="shared" ca="1" si="0"/>
+        <v>45803</v>
+      </c>
+      <c r="L6" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="M6" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="N6" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="O6" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="P6" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q6" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="R6" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="S6" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="T6" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="U6" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="V6" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="W6" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="X6" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y6" s="20">
+        <f t="shared" ca="1" si="7"/>
+        <v>45803</v>
+      </c>
+      <c r="Z6" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA6" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB6" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="AC6" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD6" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE6" s="21">
+        <v>846</v>
+      </c>
+      <c r="AF6" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG6" s="30">
+        <v>40</v>
+      </c>
+      <c r="AH6" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="AI6" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ6" s="32">
+        <f ca="1">TODAY()+365</f>
+        <v>46199</v>
+      </c>
+      <c r="AK6" s="32">
+        <f t="shared" ca="1" si="8"/>
+        <v>45893</v>
+      </c>
+      <c r="AL6" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="AM6" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="AN6" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO6" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="AP6" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="AQ6" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR6" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="AS6" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="AT6" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AU6" s="34" t="str">
+        <f>AB6</f>
+        <v>Fixed Term (Fixed Term)</v>
+      </c>
+      <c r="AV6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW6" s="35">
+        <f t="shared" ca="1" si="9"/>
+        <v>45802</v>
+      </c>
+      <c r="AX6" s="35">
+        <f t="shared" ca="1" si="10"/>
+        <v>45802</v>
+      </c>
+      <c r="AY6" s="36">
+        <f t="shared" ca="1" si="11"/>
+        <v>46199</v>
+      </c>
+      <c r="AZ6" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA6" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="BB6" s="37" t="s">
+        <v>175</v>
+      </c>
+      <c r="BC6" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="BD6" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="BE6" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF6" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="BG6" s="38">
+        <v>5555005404</v>
+      </c>
+      <c r="BH6" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BI6" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BJ6" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK6" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="BL6" s="39">
+        <v>32875</v>
+      </c>
+      <c r="BM6" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="BN6" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="BO6" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP6" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ6" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="BR6" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BS6" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="BT6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="BU6" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV6" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="BW6" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="BX6" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="BY6" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="BZ6" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="CA6" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="CB6" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="CC6" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD6" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="CE6" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF6" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CG6" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH6" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CI6" s="43">
+        <v>100</v>
+      </c>
+      <c r="CJ6" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK6" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="CL6" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="CM6" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="CN6" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="CO6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CP6" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="CQ6" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="CR6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CS6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CT6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CU6" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="CV6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:101" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="K7" s="20">
+        <f t="shared" ca="1" si="0"/>
+        <v>45803</v>
+      </c>
+      <c r="L7" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="M7" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="N7" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="O7" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="P7" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q7" s="19">
+        <v>123</v>
+      </c>
+      <c r="R7" s="19">
+        <v>1046</v>
+      </c>
+      <c r="S7" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="T7" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="U7" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="V7" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="W7" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="X7" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y7" s="20">
+        <f t="shared" ca="1" si="7"/>
+        <v>45803</v>
+      </c>
+      <c r="Z7" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA7" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB7" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="AC7" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="AD7" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE7" s="21">
+        <v>846</v>
+      </c>
+      <c r="AF7" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG7" s="30">
+        <v>10</v>
+      </c>
+      <c r="AH7" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="AI7" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ7" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="AK7" s="32">
+        <f t="shared" ca="1" si="8"/>
+        <v>45893</v>
+      </c>
+      <c r="AL7" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="AM7" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN7" s="41" t="s">
+        <v>163</v>
+      </c>
+      <c r="AO7" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="AP7" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="AQ7" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR7" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="AS7" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="AT7" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AU7" s="33" t="str">
+        <f t="shared" ref="AU7" si="13">AB7</f>
+        <v>Permanent</v>
+      </c>
+      <c r="AV7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW7" s="35">
+        <f t="shared" ca="1" si="9"/>
+        <v>45802</v>
+      </c>
+      <c r="AX7" s="35">
+        <f t="shared" ca="1" si="10"/>
+        <v>45802</v>
+      </c>
+      <c r="AY7" s="48" t="str">
+        <f t="shared" si="11"/>
+        <v>N/A</v>
+      </c>
+      <c r="AZ7" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA7" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="BB7" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="BC7" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BD7" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BE7" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF7" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="BG7" s="38">
+        <v>5555005405</v>
+      </c>
+      <c r="BH7" s="26">
+        <v>36526</v>
+      </c>
+      <c r="BI7" s="26">
+        <v>51136</v>
+      </c>
+      <c r="BJ7" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK7" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="BL7" s="39">
+        <v>32875</v>
+      </c>
+      <c r="BM7" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="BN7" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="BO7" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP7" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ7" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="BR7" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="BS7" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="BT7" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="BU7" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV7" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="BW7" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="BX7" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="BY7" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="BZ7" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="CA7" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="CB7" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="CC7" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="CD7" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="CE7" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="CF7" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CG7" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="CH7" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="CI7" s="43">
+        <v>100</v>
+      </c>
+      <c r="CJ7" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="CK7" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="CL7" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="CM7" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="CN7" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="CO7" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="CP7" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="CQ7" s="44" t="s">
+        <v>111</v>
+      </c>
+      <c r="CR7" s="50">
+        <v>31048</v>
+      </c>
+      <c r="CS7" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="CT7" s="43">
+        <v>1234011</v>
+      </c>
+      <c r="CU7" s="43">
+        <v>123456011</v>
+      </c>
+      <c r="CV7" s="43">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="13">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2">
+  <phoneticPr fontId="7" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2 Z2 X2 U2 I2:J2 CC2:CC7 BW2 AV4 Z4 X4 U4 I4:J4 BW4 AV6 Z6 X6 U6 I6:J6 BW6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($C2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV3">
-      <formula1>INDIRECT($E3)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW3">
-      <formula1>INDIRECT($E3)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC3">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:J3">
-      <formula1>INDIRECT($E3)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3">
-      <formula1>INDIRECT($E3)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X3">
-      <formula1>INDIRECT($E3)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2">
-      <formula1>INDIRECT($C2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV3 Z3 X3 U3 I3:J3 BW3 AV5 Z5 X5 U5 I5:J5 BW5 AV7 Z7 X7 U7 I7:J7 BW7" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($E3)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="W2" r:id="rId1"/>
-    <hyperlink ref="W3" r:id="rId2"/>
+    <hyperlink ref="W2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="W3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="W4" r:id="rId3" xr:uid="{212574F2-90BA-4EC3-9FF0-1A66B7682BB2}"/>
+    <hyperlink ref="W5" r:id="rId4" xr:uid="{8F08755A-B2BC-49FA-8B57-C44461772D49}"/>
+    <hyperlink ref="W6" r:id="rId5" xr:uid="{B5A90B36-9EF6-49B0-A55A-86D19CDADC5D}"/>
+    <hyperlink ref="W7" r:id="rId6" xr:uid="{3D7A8BD4-4E58-4004-BAD2-437B0C3D583D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>